<commit_message>
Add demo.ipynb, skills and copilot-instructions
</commit_message>
<xml_diff>
--- a/tests/test_data_parse/tbl1_survey.xlsx
+++ b/tests/test_data_parse/tbl1_survey.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\Box Sync\Projects\Python_ProjTables\tests\test_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\Library\CloudStorage\Box-Box\Projects\Python_Modeling_Toolbox\tests\test_data_parse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A31A14C2-719D-464E-8549-5DAD790907AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB52604D-4FB7-4C67-AFC5-6F28B67B61C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="735" yWindow="735" windowWidth="28800" windowHeight="11332" xr2:uid="{0EE3CDFA-1153-4088-A8D0-88624F64512D}"/>
+    <workbookView xWindow="1440" yWindow="1440" windowWidth="13380" windowHeight="13403" xr2:uid="{0EE3CDFA-1153-4088-A8D0-88624F64512D}"/>
   </bookViews>
   <sheets>
     <sheet name="raw_table" sheetId="1" r:id="rId1"/>
@@ -495,7 +495,7 @@
   <dimension ref="A1:D28"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="63.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.9296875" customWidth="1"/>
     <col min="2" max="2" width="14.796875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.265625" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>